<commit_message>
Add KiCad PCB design and enhance firmware
</commit_message>
<xml_diff>
--- a/calibration/WaterColumnCalibration.xlsx
+++ b/calibration/WaterColumnCalibration.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -102,12 +102,18 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -149,15 +155,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -173,8 +179,114 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -225,22 +337,22 @@
         <f aca="false">E4/F3</f>
         <v>1.72884464263916E-006</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="G4" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F5" s="0" t="n">
+      <c r="F5" s="1" t="n">
         <f aca="false">(G32-F4)/F4</f>
         <v>0.0354989348811774</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="G5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H5" s="0" t="n">
+      <c r="H5" s="1" t="n">
         <v>120</v>
       </c>
-      <c r="I5" s="0" t="n">
+      <c r="I5" s="1" t="n">
         <f aca="false">H5+F5*H5</f>
         <v>124.259872185741</v>
       </c>
@@ -293,7 +405,7 @@
         <f aca="false">C8*0.0735559</f>
         <v>94.93400288625</v>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="E8" s="1" t="n">
         <f aca="false">C8*0.001422334</f>
         <v>1.835717597925</v>
       </c>
@@ -586,7 +698,7 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G29" s="0" t="s">
+      <c r="G29" s="1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -625,10 +737,10 @@
         <f aca="false">B31-B30</f>
         <v>1248000</v>
       </c>
-      <c r="G31" s="0" t="s">
+      <c r="G31" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H31" s="0" t="s">
+      <c r="H31" s="1" t="s">
         <v>13</v>
       </c>
     </row>
@@ -655,7 +767,7 @@
         <f aca="false">E32/F31</f>
         <v>1.7947849224359E-006</v>
       </c>
-      <c r="G32" s="2" t="n">
+      <c r="G32" s="3" t="n">
         <f aca="false">AVERAGE(F32,F28,F24,F20,F16,F12,F8)</f>
         <v>1.79021678602788E-006</v>
       </c>

</xml_diff>